<commit_message>
Add generate-work-done-date-based.js script to identify hidden work
- Created new script to capture ALL work completed during sprint window
- Identifies 'hidden work' not formally assigned to sprint (21.9% of work!)
- Breaks down by issue type: Stories, Bugs, Tasks, Sub-tasks, Sub-bugs
- Calculates story points for sprint-assigned vs hidden work
- Added npm script: 'work-date-based'
- Updated README with full documentation and use cases
- Updated Sprint Health Check workflow to include hidden work analysis
- Fixed sub-bug-summary.js date-based filtering logic
</commit_message>
<xml_diff>
--- a/data/NH Story Point Plan.xlsx
+++ b/data/NH Story Point Plan.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11109"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B512F82D-4457-0040-BF3A-E394132D1ECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E63443A-CE0B-F94C-9D0F-871C9FB2F6D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Full-Delivery" sheetId="1" r:id="rId1"/>
@@ -794,17 +794,20 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="13">
@@ -4704,7 +4707,9 @@
       <c r="G3" s="9">
         <v>19</v>
       </c>
-      <c r="H3" s="9"/>
+      <c r="H3" s="9">
+        <v>11</v>
+      </c>
       <c r="I3" s="9"/>
       <c r="J3" s="9"/>
       <c r="K3" s="9"/>

</xml_diff>

<commit_message>
Populate individual sprint sheets with actual daily JIRA data from Nov 6 onwards
- Fetch actual completion data for Sprint 31 (119 pts across 12 days)
- Fetch actual completion data for Sprint 32 (6 pts on Day 1)
- Fill 'Story Points Delivered' row in each sprint sheet with real data
- Progress sheet shows current sprint (Sprint 32) with formulas
- Historical data preserved in individual sprint sheets
- Automatic detection of sprints from Nov 6, 2025 onwards
</commit_message>
<xml_diff>
--- a/data/NH Story Point Plan.xlsx
+++ b/data/NH Story Point Plan.xlsx
@@ -6113,38 +6113,42 @@
         <v>69</v>
       </c>
       <c r="B24" s="47">
-        <v>7.6</v>
+        <v>13</v>
       </c>
       <c r="C24" s="47">
-        <v>7.6</v>
-      </c>
-      <c r="D24" s="47"/>
+        <v>22</v>
+      </c>
+      <c r="D24" s="47">
+        <v>3</v>
+      </c>
       <c r="E24" s="47"/>
       <c r="F24" s="47">
-        <v>7.6</v>
+        <v>9</v>
       </c>
       <c r="G24" s="47">
-        <v>7.6</v>
+        <v>19</v>
       </c>
       <c r="H24" s="47">
-        <v>7.6</v>
+        <v>11</v>
       </c>
       <c r="I24" s="47">
-        <v>7.6</v>
+        <v>8</v>
       </c>
       <c r="J24" s="47">
-        <v>7.6</v>
-      </c>
-      <c r="K24" s="47"/>
+        <v>4</v>
+      </c>
+      <c r="K24" s="47">
+        <v>1</v>
+      </c>
       <c r="L24" s="47"/>
       <c r="M24" s="47">
-        <v>7.6</v>
+        <v>10</v>
       </c>
       <c r="N24" s="47">
-        <v>7.6</v>
+        <v>4</v>
       </c>
       <c r="O24" s="47">
-        <v>7.6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="26" spans="1:15" s="48" customFormat="1" x14ac:dyDescent="0.25">
@@ -6969,9 +6973,12 @@
         <v>23.9</v>
       </c>
     </row>
-    <row r="19" spans="1:1" s="47" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" s="47" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="47" t="s">
         <v>69</v>
+      </c>
+      <c r="B19" s="47">
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:15" s="48" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fill Progress sheet with continuous timeline from Nov 6 onwards
- Build daily points map across all sprints from Nov 6
- Fill Actual Story Points row (row 3) with continuous data
- Add Cumulative Actual formulas (row 5) for running totals
- Add Variance formulas (row 6) for planned vs actual
- Shows 15 days: Nov 6 to Nov 20 (125 total points)
- Combines Sprint 31 and Sprint 32 into unified timeline
</commit_message>
<xml_diff>
--- a/data/NH Story Point Plan.xlsx
+++ b/data/NH Story Point Plan.xlsx
@@ -3638,15 +3638,19 @@
         <v>82</v>
       </c>
       <c r="B3" s="9">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C3" s="9">
-        <v>18</v>
-      </c>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
+        <v>22</v>
+      </c>
+      <c r="D3" s="9">
+        <v>3</v>
+      </c>
+      <c r="E3" s="9">
+        <v>0</v>
+      </c>
       <c r="F3" s="9">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="G3" s="9">
         <v>19</v>
@@ -3654,14 +3658,30 @@
       <c r="H3" s="9">
         <v>11</v>
       </c>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9"/>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-      <c r="M3" s="9"/>
-      <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="9"/>
+      <c r="I3" s="9">
+        <v>8</v>
+      </c>
+      <c r="J3" s="9">
+        <v>4</v>
+      </c>
+      <c r="K3" s="9">
+        <v>1</v>
+      </c>
+      <c r="L3" s="9">
+        <v>0</v>
+      </c>
+      <c r="M3" s="9">
+        <v>10</v>
+      </c>
+      <c r="N3" s="9">
+        <v>4</v>
+      </c>
+      <c r="O3" s="9">
+        <v>15</v>
+      </c>
+      <c r="P3" s="9">
+        <v>6</v>
+      </c>
       <c r="Q3" s="9"/>
       <c r="R3" s="9"/>
       <c r="S3" s="9"/>
@@ -3833,46 +3853,46 @@
         <f>SUM($B$3:B$3)</f>
       </c>
       <c r="C5" s="9">
-        <v>37</v>
+        <f>SUM($B$3:C$3)</f>
       </c>
       <c r="D5" s="9">
-        <v>37</v>
+        <f>SUM($B$3:D$3)</f>
       </c>
       <c r="E5" s="9">
-        <v>37</v>
+        <f>SUM($B$3:E$3)</f>
       </c>
       <c r="F5" s="9">
-        <v>55</v>
+        <f>SUM($B$3:F$3)</f>
       </c>
       <c r="G5" s="9">
-        <v>74</v>
+        <f>SUM($B$3:G$3)</f>
       </c>
       <c r="H5" s="9">
-        <v>74</v>
+        <f>SUM($B$3:H$3)</f>
       </c>
       <c r="I5" s="9">
-        <v>74</v>
+        <f>SUM($B$3:I$3)</f>
       </c>
       <c r="J5" s="9">
-        <v>74</v>
+        <f>SUM($B$3:J$3)</f>
       </c>
       <c r="K5" s="9">
-        <v>74</v>
+        <f>SUM($B$3:K$3)</f>
       </c>
       <c r="L5" s="9">
-        <v>74</v>
+        <f>SUM($B$3:L$3)</f>
       </c>
       <c r="M5" s="9">
-        <v>74</v>
+        <f>SUM($B$3:M$3)</f>
       </c>
       <c r="N5" s="9">
-        <v>74</v>
+        <f>SUM($B$3:N$3)</f>
       </c>
       <c r="O5" s="9">
-        <v>74</v>
+        <f>SUM($B$3:O$3)</f>
       </c>
       <c r="P5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:P$3)</f>
       </c>
       <c r="Q5" s="42">
         <v>74</v>
@@ -3967,29 +3987,47 @@
         <f>B$4-B$5</f>
       </c>
       <c r="C6" s="9">
-        <v>7</v>
+        <f>C$4-C$5</f>
       </c>
       <c r="D6" s="9">
-        <v>7</v>
+        <f>D$4-D$5</f>
       </c>
       <c r="E6" s="9">
-        <v>7</v>
+        <f>E$4-E$5</f>
       </c>
       <c r="F6" s="9">
-        <v>0</v>
+        <f>F$4-F$5</f>
       </c>
       <c r="G6" s="9">
-        <v>-11</v>
-      </c>
-      <c r="H6" s="9"/>
-      <c r="I6" s="9"/>
-      <c r="J6" s="9"/>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="9"/>
-      <c r="O6" s="9"/>
-      <c r="P6" s="42"/>
+        <f>G$4-G$5</f>
+      </c>
+      <c r="H6" s="9">
+        <f>H$4-H$5</f>
+      </c>
+      <c r="I6" s="9">
+        <f>I$4-I$5</f>
+      </c>
+      <c r="J6" s="9">
+        <f>J$4-J$5</f>
+      </c>
+      <c r="K6" s="9">
+        <f>K$4-K$5</f>
+      </c>
+      <c r="L6" s="9">
+        <f>L$4-L$5</f>
+      </c>
+      <c r="M6" s="9">
+        <f>M$4-M$5</f>
+      </c>
+      <c r="N6" s="9">
+        <f>N$4-N$5</f>
+      </c>
+      <c r="O6" s="9">
+        <f>O$4-O$5</f>
+      </c>
+      <c r="P6" s="42">
+        <f>P$4-P$5</f>
+      </c>
       <c r="Q6" s="42"/>
       <c r="R6" s="42"/>
       <c r="S6" s="42"/>
@@ -6121,7 +6159,9 @@
       <c r="D24" s="47">
         <v>3</v>
       </c>
-      <c r="E24" s="47"/>
+      <c r="E24" s="47">
+        <v>0</v>
+      </c>
       <c r="F24" s="47">
         <v>9</v>
       </c>
@@ -6140,7 +6180,9 @@
       <c r="K24" s="47">
         <v>1</v>
       </c>
-      <c r="L24" s="47"/>
+      <c r="L24" s="47">
+        <v>0</v>
+      </c>
       <c r="M24" s="47">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Change generate-sheets to use date-based completion like work-done
- Query ALL issues completed on each date, not filtered by sprint
- Matches work-done-today logic exactly
- Nov 6-19: 152 points (was 119 when sprint-filtered)
- Nov 20: 33 points (was 6 when sprint-filtered)
- Total: 185 points (was 125)
- More accurate representation of actual daily velocity
- Captures work completed regardless of sprint assignment
</commit_message>
<xml_diff>
--- a/data/NH Story Point Plan.xlsx
+++ b/data/NH Story Point Plan.xlsx
@@ -3638,10 +3638,10 @@
         <v>82</v>
       </c>
       <c r="B3" s="9">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C3" s="9">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D3" s="9">
         <v>3</v>
@@ -3656,13 +3656,13 @@
         <v>19</v>
       </c>
       <c r="H3" s="9">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I3" s="9">
         <v>8</v>
       </c>
       <c r="J3" s="9">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K3" s="9">
         <v>1</v>
@@ -3671,16 +3671,16 @@
         <v>0</v>
       </c>
       <c r="M3" s="9">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="N3" s="9">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="O3" s="9">
         <v>15</v>
       </c>
       <c r="P3" s="9">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="Q3" s="9"/>
       <c r="R3" s="9"/>
@@ -6151,10 +6151,10 @@
         <v>69</v>
       </c>
       <c r="B24" s="47">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C24" s="47">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D24" s="47">
         <v>3</v>
@@ -6169,13 +6169,13 @@
         <v>19</v>
       </c>
       <c r="H24" s="47">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I24" s="47">
         <v>8</v>
       </c>
       <c r="J24" s="47">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K24" s="47">
         <v>1</v>
@@ -6184,10 +6184,10 @@
         <v>0</v>
       </c>
       <c r="M24" s="47">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="N24" s="47">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="O24" s="47">
         <v>15</v>
@@ -7020,7 +7020,7 @@
         <v>69</v>
       </c>
       <c r="B19" s="47">
-        <v>6</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:15" s="48" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Add daily flow metrics, sprint health, overall plan health, and Jira reporting scripts
- Daily flow metrics with team-grouped Entry SP, grid tables
- Sprint health and overall plan health reports
- Align sprint health with daily flow (same sprint ID, matching Done totals)
- Open QA defects by assignee, completed 2A, done rate, SP left
- Fix version update, release progress, workflow queue metrics
- FR analysis, delivery analysis, productivity reports
- Additional data files and analysis outputs

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/NH Story Point Plan.xlsx
+++ b/data/NH Story Point Plan.xlsx
@@ -3562,38 +3562,38 @@
         <v>12.5</v>
       </c>
       <c r="P2" s="40">
-        <v>13.6</v>
+        <v>12</v>
       </c>
       <c r="Q2" s="40">
-        <v>19</v>
+        <v>16.7</v>
       </c>
       <c r="R2" s="40"/>
       <c r="S2" s="40"/>
       <c r="T2" s="40">
-        <v>27.1</v>
+        <v>23.9</v>
       </c>
       <c r="U2" s="40">
-        <v>32.5</v>
+        <v>28.7</v>
       </c>
       <c r="V2" s="40">
-        <v>35.2</v>
+        <v>31.1</v>
       </c>
       <c r="W2" s="40">
-        <v>51.5</v>
+        <v>45.4</v>
       </c>
       <c r="X2" s="40">
-        <v>32.5</v>
+        <v>28.7</v>
       </c>
       <c r="Y2" s="40"/>
       <c r="Z2" s="40"/>
       <c r="AA2" s="40">
-        <v>27.1</v>
+        <v>23.9</v>
       </c>
       <c r="AB2" s="40">
-        <v>19</v>
+        <v>16.7</v>
       </c>
       <c r="AC2" s="40">
-        <v>13.6</v>
+        <v>12</v>
       </c>
       <c r="AD2" s="40">
         <v>12.4</v>
@@ -3641,7 +3641,7 @@
         <v>19</v>
       </c>
       <c r="C3" s="9">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D3" s="9">
         <v>3</v>
@@ -3682,27 +3682,69 @@
       <c r="P3" s="9">
         <v>33</v>
       </c>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="9"/>
-      <c r="S3" s="9"/>
-      <c r="T3" s="9"/>
-      <c r="U3" s="9"/>
-      <c r="V3" s="9"/>
-      <c r="W3" s="9"/>
-      <c r="X3" s="9"/>
-      <c r="Y3" s="9"/>
-      <c r="Z3" s="9"/>
-      <c r="AA3" s="9"/>
-      <c r="AB3" s="9"/>
-      <c r="AC3" s="9"/>
-      <c r="AD3" s="9"/>
-      <c r="AE3" s="9"/>
-      <c r="AF3" s="9"/>
-      <c r="AG3" s="9"/>
-      <c r="AH3" s="9"/>
-      <c r="AI3" s="9"/>
-      <c r="AJ3" s="9"/>
-      <c r="AK3" s="9"/>
+      <c r="Q3" s="9">
+        <v>10</v>
+      </c>
+      <c r="R3" s="9">
+        <v>0</v>
+      </c>
+      <c r="S3" s="9">
+        <v>0</v>
+      </c>
+      <c r="T3" s="9">
+        <v>4</v>
+      </c>
+      <c r="U3" s="9">
+        <v>18</v>
+      </c>
+      <c r="V3" s="9">
+        <v>14</v>
+      </c>
+      <c r="W3" s="9">
+        <v>18</v>
+      </c>
+      <c r="X3" s="9">
+        <v>26</v>
+      </c>
+      <c r="Y3" s="9">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="9">
+        <v>0</v>
+      </c>
+      <c r="AA3" s="9">
+        <v>22.5</v>
+      </c>
+      <c r="AB3" s="9">
+        <v>22</v>
+      </c>
+      <c r="AC3" s="9">
+        <v>20</v>
+      </c>
+      <c r="AD3" s="9">
+        <v>31.5</v>
+      </c>
+      <c r="AE3" s="9">
+        <v>27</v>
+      </c>
+      <c r="AF3" s="9">
+        <v>3</v>
+      </c>
+      <c r="AG3" s="9">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="9">
+        <v>19</v>
+      </c>
+      <c r="AI3" s="9">
+        <v>9</v>
+      </c>
+      <c r="AJ3" s="9">
+        <v>9</v>
+      </c>
+      <c r="AK3" s="9">
+        <v>21</v>
+      </c>
       <c r="AL3" s="9"/>
       <c r="AM3" s="9"/>
       <c r="AN3" s="9"/>
@@ -3758,91 +3800,91 @@
         <v>250</v>
       </c>
       <c r="P4" s="42">
-        <v>263.6</v>
+        <v>262</v>
       </c>
       <c r="Q4" s="42">
-        <v>282.6</v>
+        <v>278.7</v>
       </c>
       <c r="R4" s="42">
-        <v>282.6</v>
+        <v>278.7</v>
       </c>
       <c r="S4" s="42">
-        <v>282.6</v>
+        <v>278.7</v>
       </c>
       <c r="T4" s="42">
-        <v>309.7</v>
+        <v>302.6</v>
       </c>
       <c r="U4" s="42">
-        <v>342.2</v>
+        <v>331.3</v>
       </c>
       <c r="V4" s="42">
-        <v>377.4</v>
+        <v>362.4</v>
       </c>
       <c r="W4" s="42">
-        <v>428.9</v>
+        <v>407.8</v>
       </c>
       <c r="X4" s="42">
-        <v>461.4</v>
+        <v>436.5</v>
       </c>
       <c r="Y4" s="42">
-        <v>461.4</v>
+        <v>436.5</v>
       </c>
       <c r="Z4" s="42">
-        <v>461.4</v>
+        <v>436.5</v>
       </c>
       <c r="AA4" s="42">
-        <v>488.5</v>
+        <v>460.4</v>
       </c>
       <c r="AB4" s="42">
-        <v>507.5</v>
+        <v>477.1</v>
       </c>
       <c r="AC4" s="42">
-        <v>521.1</v>
+        <v>489.1</v>
       </c>
       <c r="AD4" s="42">
-        <v>533.5</v>
+        <v>501.5</v>
       </c>
       <c r="AE4" s="42">
-        <v>550.9</v>
+        <v>518.9</v>
       </c>
       <c r="AF4" s="42">
-        <v>550.9</v>
+        <v>518.9</v>
       </c>
       <c r="AG4" s="42">
-        <v>550.9</v>
+        <v>518.9</v>
       </c>
       <c r="AH4" s="42">
-        <v>575.7</v>
+        <v>543.7</v>
       </c>
       <c r="AI4" s="42">
-        <v>605.5</v>
+        <v>573.5</v>
       </c>
       <c r="AJ4" s="42">
-        <v>637.7</v>
+        <v>605.7</v>
       </c>
       <c r="AK4" s="42">
-        <v>684.8</v>
+        <v>652.8</v>
       </c>
       <c r="AL4" s="42">
-        <v>714.6</v>
+        <v>682.6</v>
       </c>
       <c r="AM4" s="42">
-        <v>714.6</v>
+        <v>682.6</v>
       </c>
       <c r="AN4" s="42">
-        <v>714.6</v>
+        <v>682.6</v>
       </c>
       <c r="AO4" s="42">
-        <v>739.4</v>
+        <v>707.4</v>
       </c>
       <c r="AP4" s="42">
-        <v>756.8</v>
+        <v>724.8</v>
       </c>
       <c r="AQ4" s="42">
-        <v>769.2</v>
+        <v>737.2</v>
       </c>
       <c r="AR4" s="42">
-        <v>777.9</v>
+        <v>745.9</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.25">
@@ -3895,88 +3937,88 @@
         <f>SUM($B$3:P$3)</f>
       </c>
       <c r="Q5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:Q$3)</f>
       </c>
       <c r="R5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:R$3)</f>
       </c>
       <c r="S5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:S$3)</f>
       </c>
       <c r="T5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:T$3)</f>
       </c>
       <c r="U5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:U$3)</f>
       </c>
       <c r="V5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:V$3)</f>
       </c>
       <c r="W5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:W$3)</f>
       </c>
       <c r="X5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:X$3)</f>
       </c>
       <c r="Y5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:Y$3)</f>
       </c>
       <c r="Z5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:Z$3)</f>
       </c>
       <c r="AA5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:[$3)</f>
       </c>
       <c r="AB5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:\$3)</f>
       </c>
       <c r="AC5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:]$3)</f>
       </c>
       <c r="AD5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:^$3)</f>
       </c>
       <c r="AE5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:_$3)</f>
       </c>
       <c r="AF5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:`$3)</f>
       </c>
       <c r="AG5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:a$3)</f>
       </c>
       <c r="AH5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:b$3)</f>
       </c>
       <c r="AI5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:c$3)</f>
       </c>
       <c r="AJ5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:d$3)</f>
       </c>
       <c r="AK5" s="42">
-        <v>74</v>
+        <f>SUM($B$3:e$3)</f>
       </c>
       <c r="AL5" s="42">
-        <v>74</v>
+        <v>374.5</v>
       </c>
       <c r="AM5" s="42">
-        <v>74</v>
+        <v>374.5</v>
       </c>
       <c r="AN5" s="42">
-        <v>74</v>
+        <v>374.5</v>
       </c>
       <c r="AO5" s="42">
-        <v>74</v>
+        <v>374.5</v>
       </c>
       <c r="AP5" s="42">
-        <v>74</v>
+        <v>374.5</v>
       </c>
       <c r="AQ5" s="42">
-        <v>74</v>
+        <v>374.5</v>
       </c>
       <c r="AR5" s="42">
-        <v>74</v>
+        <v>374.5</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.25">
@@ -4028,27 +4070,69 @@
       <c r="P6" s="42">
         <f>P$4-P$5</f>
       </c>
-      <c r="Q6" s="42"/>
-      <c r="R6" s="42"/>
-      <c r="S6" s="42"/>
-      <c r="T6" s="42"/>
-      <c r="U6" s="42"/>
-      <c r="V6" s="42"/>
-      <c r="W6" s="42"/>
-      <c r="X6" s="42"/>
-      <c r="Y6" s="42"/>
-      <c r="Z6" s="42"/>
-      <c r="AA6" s="42"/>
-      <c r="AB6" s="42"/>
-      <c r="AC6" s="42"/>
-      <c r="AD6" s="42"/>
-      <c r="AE6" s="42"/>
-      <c r="AF6" s="42"/>
-      <c r="AG6" s="42"/>
-      <c r="AH6" s="42"/>
-      <c r="AI6" s="42"/>
-      <c r="AJ6" s="42"/>
-      <c r="AK6" s="42"/>
+      <c r="Q6" s="42">
+        <f>Q$4-Q$5</f>
+      </c>
+      <c r="R6" s="42">
+        <f>R$4-R$5</f>
+      </c>
+      <c r="S6" s="42">
+        <f>S$4-S$5</f>
+      </c>
+      <c r="T6" s="42">
+        <f>T$4-T$5</f>
+      </c>
+      <c r="U6" s="42">
+        <f>U$4-U$5</f>
+      </c>
+      <c r="V6" s="42">
+        <f>V$4-V$5</f>
+      </c>
+      <c r="W6" s="42">
+        <f>W$4-W$5</f>
+      </c>
+      <c r="X6" s="42">
+        <f>X$4-X$5</f>
+      </c>
+      <c r="Y6" s="42">
+        <f>Y$4-Y$5</f>
+      </c>
+      <c r="Z6" s="42">
+        <f>Z$4-Z$5</f>
+      </c>
+      <c r="AA6" s="42">
+        <f>[$4-[$5</f>
+      </c>
+      <c r="AB6" s="42">
+        <f>\$4-\$5</f>
+      </c>
+      <c r="AC6" s="42">
+        <f>]$4-]$5</f>
+      </c>
+      <c r="AD6" s="42">
+        <f>^$4-^$5</f>
+      </c>
+      <c r="AE6" s="42">
+        <f>_$4-_$5</f>
+      </c>
+      <c r="AF6" s="42">
+        <f>`$4-`$5</f>
+      </c>
+      <c r="AG6" s="42">
+        <f>a$4-a$5</f>
+      </c>
+      <c r="AH6" s="42">
+        <f>b$4-b$5</f>
+      </c>
+      <c r="AI6" s="42">
+        <f>c$4-c$5</f>
+      </c>
+      <c r="AJ6" s="42">
+        <f>d$4-d$5</f>
+      </c>
+      <c r="AK6" s="42">
+        <f>e$4-e$5</f>
+      </c>
       <c r="AL6" s="42"/>
       <c r="AM6" s="42"/>
       <c r="AN6" s="42"/>
@@ -4062,133 +4146,133 @@
         <v>86</v>
       </c>
       <c r="B7" s="9">
-        <v>750</v>
+        <v>718</v>
       </c>
       <c r="C7" s="9">
-        <v>732</v>
+        <v>692</v>
       </c>
       <c r="D7" s="9">
-        <v>732</v>
+        <v>689</v>
       </c>
       <c r="E7" s="9">
-        <v>732</v>
+        <v>689</v>
       </c>
       <c r="F7" s="9">
-        <v>714</v>
+        <v>680</v>
       </c>
       <c r="G7" s="9">
-        <v>695</v>
+        <v>661</v>
       </c>
       <c r="H7" s="9">
-        <v>695</v>
+        <v>635</v>
       </c>
       <c r="I7" s="9">
-        <v>695</v>
+        <v>627</v>
       </c>
       <c r="J7" s="9">
-        <v>695</v>
+        <v>620</v>
       </c>
       <c r="K7" s="9">
-        <v>695</v>
+        <v>619</v>
       </c>
       <c r="L7" s="9">
-        <v>695</v>
+        <v>619</v>
       </c>
       <c r="M7" s="9">
-        <v>695</v>
+        <v>606</v>
       </c>
       <c r="N7" s="9">
-        <v>695</v>
+        <v>598</v>
       </c>
       <c r="O7" s="9">
-        <v>695</v>
+        <v>583</v>
       </c>
       <c r="P7" s="42">
-        <v>695</v>
+        <v>550</v>
       </c>
       <c r="Q7" s="42">
-        <v>695</v>
+        <v>540</v>
       </c>
       <c r="R7" s="42">
-        <v>695</v>
+        <v>540</v>
       </c>
       <c r="S7" s="42">
-        <v>695</v>
+        <v>540</v>
       </c>
       <c r="T7" s="42">
-        <v>695</v>
+        <v>536</v>
       </c>
       <c r="U7" s="42">
-        <v>695</v>
+        <v>518</v>
       </c>
       <c r="V7" s="42">
-        <v>695</v>
+        <v>504</v>
       </c>
       <c r="W7" s="42">
-        <v>695</v>
+        <v>486</v>
       </c>
       <c r="X7" s="42">
-        <v>695</v>
+        <v>458</v>
       </c>
       <c r="Y7" s="42">
-        <v>695</v>
+        <v>458</v>
       </c>
       <c r="Z7" s="42">
-        <v>695</v>
+        <v>458</v>
       </c>
       <c r="AA7" s="42">
-        <v>695</v>
+        <v>435.5</v>
       </c>
       <c r="AB7" s="42">
-        <v>695</v>
+        <v>408.5</v>
       </c>
       <c r="AC7" s="42">
-        <v>695</v>
+        <v>388.5</v>
       </c>
       <c r="AD7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AE7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AF7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AG7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AH7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AI7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AJ7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AK7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AL7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AM7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AN7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AO7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AP7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AQ7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
       <c r="AR7" s="42">
-        <v>695</v>
+        <v>362.5</v>
       </c>
     </row>
   </sheetData>
@@ -6154,7 +6238,7 @@
         <v>19</v>
       </c>
       <c r="C24" s="47">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D24" s="47">
         <v>3</v>
@@ -7015,12 +7099,51 @@
         <v>23.9</v>
       </c>
     </row>
-    <row r="19" spans="1:2" s="47" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" s="47" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="47" t="s">
         <v>69</v>
       </c>
       <c r="B19" s="47">
-        <v>33</v>
+        <v>31</v>
+      </c>
+      <c r="C19" s="47">
+        <v>10</v>
+      </c>
+      <c r="D19" s="47">
+        <v>0</v>
+      </c>
+      <c r="E19" s="47">
+        <v>0</v>
+      </c>
+      <c r="F19" s="47">
+        <v>4</v>
+      </c>
+      <c r="G19" s="47">
+        <v>18</v>
+      </c>
+      <c r="H19" s="47">
+        <v>14</v>
+      </c>
+      <c r="I19" s="47">
+        <v>18</v>
+      </c>
+      <c r="J19" s="47">
+        <v>28</v>
+      </c>
+      <c r="K19" s="47">
+        <v>0</v>
+      </c>
+      <c r="L19" s="47">
+        <v>0</v>
+      </c>
+      <c r="M19" s="47">
+        <v>22.5</v>
+      </c>
+      <c r="N19" s="47">
+        <v>27</v>
+      </c>
+      <c r="O19" s="47">
+        <v>20</v>
       </c>
     </row>
     <row r="21" spans="1:15" s="48" customFormat="1" x14ac:dyDescent="0.25">
@@ -7810,9 +7933,33 @@
         <v>24.799999999999997</v>
       </c>
     </row>
-    <row r="18" spans="1:1" s="47" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" s="47" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="47" t="s">
         <v>69</v>
+      </c>
+      <c r="B18" s="47">
+        <v>31.5</v>
+      </c>
+      <c r="C18" s="47">
+        <v>27</v>
+      </c>
+      <c r="D18" s="47">
+        <v>3</v>
+      </c>
+      <c r="E18" s="47">
+        <v>0</v>
+      </c>
+      <c r="F18" s="47">
+        <v>19</v>
+      </c>
+      <c r="G18" s="47">
+        <v>9</v>
+      </c>
+      <c r="H18" s="47">
+        <v>11</v>
+      </c>
+      <c r="I18" s="47">
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:15" s="48" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>